<commit_message>
Update: New Branch for 2D with 3 Anchor
</commit_message>
<xml_diff>
--- a/uwb_dashboard/recordings/rtls.xlsx
+++ b/uwb_dashboard/recordings/rtls.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +48,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,48 +437,323 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>z</t>
+          <t>A2_Range</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>A1_Range</t>
+          <t>A3_Range</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>A2_Range</t>
+          <t>A4_Range</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>A3_Range</t>
+          <t>A2_RSSI</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>A4_Range</t>
+          <t>A3_RSSI</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>A1_RSSI</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>A2_RSSI</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>A3_RSSI</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
           <t>A4_RSSI</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>45994.30595092418</v>
+      </c>
+      <c r="B2" t="n">
+        <v>807.3943999999992</v>
+      </c>
+      <c r="C2" t="n">
+        <v>-3329.98975</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-104.38</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-96.34</v>
+      </c>
+      <c r="F2" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-53.75</v>
+      </c>
+      <c r="H2" t="n">
+        <v>-54.55</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-53.64</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>45994.30596398065</v>
+      </c>
+      <c r="B3" t="n">
+        <v>3717.607749999999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-1285.36825</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-104.38</v>
+      </c>
+      <c r="E3" t="n">
+        <v>58.83</v>
+      </c>
+      <c r="F3" t="n">
+        <v>29.82</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-53.75</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-52.61</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-53.55</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>45994.30597716351</v>
+      </c>
+      <c r="B4" t="n">
+        <v>4517.99375</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-59.7364</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-104.38</v>
+      </c>
+      <c r="E4" t="n">
+        <v>43.13</v>
+      </c>
+      <c r="F4" t="n">
+        <v>41.71</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-53.75</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-53.71</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-53.58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>45994.30599013185</v>
+      </c>
+      <c r="B5" t="n">
+        <v>10985.75075</v>
+      </c>
+      <c r="C5" t="n">
+        <v>73.64999999999998</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-148.72</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="F5" t="n">
+        <v>17.13</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-54.1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-54.22</v>
+      </c>
+      <c r="I5" t="n">
+        <v>-53.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>45994.30600276821</v>
+      </c>
+      <c r="B6" t="n">
+        <v>6964.1942</v>
+      </c>
+      <c r="C6" t="n">
+        <v>-372.5057999999999</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-148.72</v>
+      </c>
+      <c r="E6" t="n">
+        <v>-90.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>86.28</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-54.1</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-52.61</v>
+      </c>
+      <c r="I6" t="n">
+        <v>-54.65</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>45994.3060153313</v>
+      </c>
+      <c r="B7" t="n">
+        <v>9202.4774</v>
+      </c>
+      <c r="C7" t="n">
+        <v>-1251.5176</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-148.72</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60.94</v>
+      </c>
+      <c r="F7" t="n">
+        <v>34.78</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-54.1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-54.31</v>
+      </c>
+      <c r="I7" t="n">
+        <v>-54.23</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>45994.30602822267</v>
+      </c>
+      <c r="B8" t="n">
+        <v>1497.257150000001</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-8346.809999999998</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-148.72</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-138.29</v>
+      </c>
+      <c r="F8" t="n">
+        <v>49.29</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-54.1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-52.16</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-54.24</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>45994.3060413584</v>
+      </c>
+      <c r="B9" t="n">
+        <v>13871.23265</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5454.45825</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-172.97</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-46.66</v>
+      </c>
+      <c r="F9" t="n">
+        <v>114.39</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-53.86</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-52.84</v>
+      </c>
+      <c r="I9" t="n">
+        <v>-54.1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>45994.30605404013</v>
+      </c>
+      <c r="B10" t="n">
+        <v>14903.0992</v>
+      </c>
+      <c r="C10" t="n">
+        <v>4381.550799999999</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-172.97</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-10.65</v>
+      </c>
+      <c r="F10" t="n">
+        <v>94.20999999999999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-53.86</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-53.15</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-54.52</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>45994.3060666628</v>
+      </c>
+      <c r="B11" t="n">
+        <v>14925.86165</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-33.23755</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-172.97</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-8.24</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.65</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-53.86</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-51.75</v>
+      </c>
+      <c r="I11" t="n">
+        <v>-54.79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>